<commit_message>
Add shop configuration dialog with URL list, live search, and add dialog
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1086,14 +1086,142 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>https://express.auchan.ua/konfety-bob-snail-jablochno-vishnevye-v-bel-gijskom-chjornom-shokolade-30-g-934001/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Мармелад натуральний Bob Snail Яблуко-вишня, 27 г</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>30,50</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Bob Snail</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/marmelad-natural-nyj-bob-snail-jabloko-vishnja-27-g-1271227/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Фоззі</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Пастила фруктова «Премія»® груша-яблуко та яблуко-персик</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>31.49 ₴</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>26.49 ₴</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Премія</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://fozzyshop.ua/skhidni-solodoshchi-khalva/950652-pastyla-fruktova-premiia-grusha-iabluko-ta-iabluko-persyk.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Варус</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Цукерки Bob Snail натуральні яблучні 60 г</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>82.90</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Bob Snail</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://varus.ua/cukerki-naturalni-yabluchni-bob-snail-60g</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>АТБ</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.atbmarket.com/product/cukerki-60g-ravlik-bob-yabluko-grusa</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add individual progress bars for each shop and centered layout
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,6 +512,886 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Мармелад натуральний Bob Snail Яблуко-вишня, 27 г</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>30,50</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/marmelad-natural-nyj-bob-snail-jabloko-vishnja-27-g-1271227/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Сільпо</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Арахіс смажений солоний, 500г</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>139.00 грн</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>84.79 грн</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Без ТМ</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://silpo.ua/product/arakhis-smazhenyi-solonyi-476739</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Батончик Bob Snail Яблуко‑вишня‑кеш'ю‑кріспи кіноа 35 г (4820287102558)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>57,70</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>43,90</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/batonchik-bob-snail-jabluko-vishnja-kesh-ju-krispi-kinoa-35-g-4820287102558-2069212/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Сільпо</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Масло солодковершкове Біло Екстра 82%, 400г</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>299.00 грн</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>159.00 грн</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Біло</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://silpo.ua/product/maslo-solodkovershkove-bilo-ekstra-82-1031734</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Цукерки Snail Bob яблучно-малинові у бельгійському чорному шоколаді, 60 г</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>84,00</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/konfety-bob-snail-jablochno-malinovye-v-bel-gijskom-chjornom-shokolade-60-g-934079/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Натуральні яблучні цукерки Bob Snail, 120 г</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>89,80</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/natural-nye-jablochnye-konfety-bob-snail-120-g-264479/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Батончик Bob Snail Хурма‑апельсин‑кеш'ю‑кріспи кіноа 35 г (4820287102596)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>57,70</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/batonchik-bob-snail-hurma-apel-sin-kesh-ju-krispi-kinoa-35-g-4820287102596-2069218/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Подарунковий бокс Bob Snail з грою та іграшкою 300 г (4820287101193)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>591,70</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/podarunkovij-boks-bob-snail-z-groju-ta-igrashkoju-300-g-4820287101193-2023602/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Пюре фруктове Груша Bob Snail д/п 400г</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>65,60</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/pjure-fruktovoe-grusha-bob-snail-d-p-400g-691755/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Пюре фруктове Смузі Груша-лісова ожина Bob Snail д/п 120г</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>29,80</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/pjure-fruktovoe-smuzi-grusha-lesnaja-ezhevika-bob-snail-d-p-120g-691811/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Цукерка Bob Snail Дооовга хурма‑ананас фруктова натуральна 15 г (4820287102442)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>24,50</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/cukerka-bob-snail-dooovga-hurma-ananas-fruktova-natural-na-15-g-4820287102442-2069329/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Набір продукції Bob Snail Подарунковий бокс Снек трек з іграшкою та стікером 107 г (4820219348665)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>389,70</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/nabir-produkcii-bob-snail-podarunkovij-boks-snek-trek-z-igrashkoju-ta-stikerom-107-g-4820219348665-1797279/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Мангове пюре дитяче Bob Snail, 400 г</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>94,80</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/mangovoe-pjure-detskoe-bob-snail-400-g-526960/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Цукерки Snail Bob яблучно-вишневі в бельгійському чорному шоколаді, 30 г</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/konfety-bob-snail-jablochno-vishnevye-v-bel-gijskom-chjornom-shokolade-30-g-934001/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Цукерки Snail Bob яблучно-грушеві в бельгійському молочному шоколаді, 30 г</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>55,90</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/konfety-bob-snail-jablochno-grushevye-v-bel-gijskom-molochnom-shokolade-30-g-934019/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Пюре фруктове Bob Snail Персик, 250 г</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>96,50</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/pjure-fruktovoe-bob-snail-persik-250-g-1174263/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Мармелад Snail Bob груша-малина-буряк без цукру, 108 г</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>104,40</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/marmelad-bob-snail-grusha-malina-svekla-bez-sahara-108-g-934127/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Мармелад Snail Bob яблуко-манго-гарбуз-чіа в бельгійському молочному шоколаді, 27 г</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>51,40</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/marmelad-bob-snail-jabloko-mango-tykva-chia-v-bel-gijskom-molochnom-shokolade-27-g-933989/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Пюре фруктове для дітей від 5 місяців Яблуко-банан Bob Snail 90 г</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>23,60</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/pjure-fruktovoe-dlja-detej-ot-5-mesjacev-jabloko-banan-bob-snail-90-g-737640-901653/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Натуральні З Хурми Страйпи Bob Snail, 14г</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>21,40</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/natural-nye-iz-hurmy-strajpy-bob-snail-14g-1236960/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Мармелад натуральний Bob Snail Яблуко-Морква, 27 г</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>27,50</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/marmelad-natural-nyj-bob-snail-jabloko-morkov-27-g-1271262/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Мармелад натуральний Bob Snail Груша-апельсин, 27 г</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>37,50</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/marmelad-natural-nyj-bob-snail-grusha-apel-sin-27-g-1271241/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Цукерки натуральні фруктові З хурми сорт Шарон Bob Snail к/у 60г</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>81,90</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/konfety-natural-nye-fruktovye-s-hurmy-sort-sharon-bob-snail-k-u-60g-680369/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Цукерка Bob Snail Дооовга яблуко‑полуниця натуральна 15 г (4820287102336)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>22,90</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/cukerka-bob-snail-dooovga-jabluko-polunicja-natural-na-15-g-4820287102336-2069320/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Пюре фруктове Смузі Манго-кокос Bob Snail д/п 120г</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>46,40</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/pjure-fruktovoe-smuzi-mango-kokos-bob-snail-d-p-120g-691818/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Мармелад Snail Bob яблуко-манго-гарбуз-чіа в бельгійському молочному шоколаді, 54 г</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>81,50</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/marmelad-bob-snail-jabloko-mango-tykva-chia-v-bel-gijskom-molochnom-shokolade-54-g-934061/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Набір цукерок Bob Snail School Box з іграшкою 231 г (4820219349488)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>317,90</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/nabir-cukerok-bob-snail-school-box-z-igrashkoju-231-g-4820219349488-1753408/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Пюре фруктово-ягідне Bob Snail Смузі Яблуко-чорна смородина від 6 місяців 120 г (4820219343790)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>46,10</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/pjure-fruktovoe-smuzi-jabloko-chernaja-smorodina-bob-snail-d-p-120g-691832/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Натуральні Страйпи яблучно-вишневі Bob Snail, 14г</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>21,20</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/natural-nye-jablochno-vishnevye-strajpy-bob-snail-14g-1236953/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Цукерки натуральні яблучно-малинові Bob Snail к/у 60г</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>74,00</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/konfety-natural-nye-jablochno-malinovye-bob-snail-k-u-60g-684769/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Цукерки в чорному шоколаді Bob Snail яблучно-малинові, 30 г</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/konfety-v-chernom-shokolade-bob-snail-jablochno-malinovye-30-g-755147/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add macro capture mode for quick URL addition via F8 and clipboard
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1381,14 +1381,330 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/konfety-v-chernom-shokolade-bob-snail-jablochno-malinovye-30-g-755147/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Натуральні цукерки Bob Snail Яблучно-Смородинові 60 г</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>92,70</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/natural-nye-konfety-bob-snail-jablochno-cmorodinovye-60-g-1236981/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Снек фруктово-ягідний Bob Snail Baby Яблуко-малина для дітей від 12-ти місяців 17 г (4820287103623)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>26,60</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/snek-fruktovo-jagidnij-bob-snail-baby-jabluko-malina-dlja-ditej-vid-12-ti-misjaciv-17-g-4820287103623-2096218/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Цукерки фруктово-ягідні натуральні Bob Snail Apple-raspberry Rolls, 100 г</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>103,70</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/cukerki-fruktovo-jagidni-natural-ni-bob-snail-apple-raspberry-rolls-100-g-1624544/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Натуральний фруктовий мармелад Bob Snail Равлик Боб Яблуко-Манго-Гарбуз-Чіа, 54 г</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>52,90</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/natural-nyj-fruktovyj-marmelad-bob-snail-ravlik-bob-jabloko-mango-tykva-chia-54-g-673688-899557/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Мармелад натуральний Bob Snail Яблуко-вишня, 27 г</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>30,50</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/marmelad-natural-nyj-bob-snail-jabloko-vishnja-27-g-1271227/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Батончик Bob Snail Яблуко‑вишня‑кеш'ю‑кріспи кіноа 35 г (4820287102558)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>57,70</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>43,90</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/batonchik-bob-snail-jabluko-vishnja-kesh-ju-krispi-kinoa-35-g-4820287102558-2069212/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Сільпо</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Арахіс смажений солоний, 500г</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>139.00 грн</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://silpo.ua/product/arakhis-smazhenyi-solonyi-476739</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Цукерки Snail Bob яблучно-малинові у бельгійському чорному шоколаді, 60 г</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>84,00</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/konfety-bob-snail-jablochno-malinovye-v-bel-gijskom-chjornom-shokolade-60-g-934079/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Натуральні яблучні цукерки Bob Snail, 120 г</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>89,80</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/natural-nye-jablochnye-konfety-bob-snail-120-g-264479/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Сільпо</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Масло солодковершкове Біло Екстра 82%, 400г</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>299.00 грн</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://silpo.ua/product/maslo-solodkovershkove-bilo-ekstra-82-1031734</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Ашан</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Батончик Bob Snail Хурма‑апельсин‑кеш'ю‑кріспи кіноа 35 г (4820287102596)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>57,70</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>NULL</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>https://express.auchan.ua/konfety-v-chernom-shokolade-bob-snail-jablochno-malinovye-30-g-755147/</t>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://express.auchan.ua/batonchik-bob-snail-hurma-apel-sin-kesh-ju-krispi-kinoa-35-g-4820287102596-2069218/</t>
         </is>
       </c>
     </row>

</xml_diff>